<commit_message>
Update for Ragas evaluation
</commit_message>
<xml_diff>
--- a/RiskHalo_Certification_Challenge/data/Weekly_Trade_Data_Uploads/Week_10_Trade_data.xlsx
+++ b/RiskHalo_Certification_Challenge/data/Weekly_Trade_Data_Uploads/Week_10_Trade_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SOFTWARES\CodeRepo\AIE9_CERTIFICATION_CHALLENGE\RiskHalo_Certification_Challenge\data\Weekly_Trade_Data_Uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83AB3240-D8FF-42FB-8CDB-E261FC0DB6B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5485547F-871D-4C35-AAEB-77422F095A6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
   <si>
     <t>Sr.</t>
   </si>
@@ -55,19 +55,37 @@
     <t>Turnover</t>
   </si>
   <si>
-    <t>OPT NIFTY 19 Jun 2025 25000 PE</t>
-  </si>
-  <si>
-    <t>17-06-2025</t>
-  </si>
-  <si>
-    <t>OPT NIFTY 19 Jun 2025 24800 CE</t>
-  </si>
-  <si>
-    <t>OPT DIVISLAB 26 Jun 2025 6600 CE</t>
-  </si>
-  <si>
-    <t>18-06-2025</t>
+    <t>OPT POLYCAB 31 Jul 2025 6900 CE</t>
+  </si>
+  <si>
+    <t>21-07-2025</t>
+  </si>
+  <si>
+    <t>OPT DALBHARAT 31 Jul 2025 2240 CE</t>
+  </si>
+  <si>
+    <t>OPT PATANJALI 31 Jul 2025 1900 PE</t>
+  </si>
+  <si>
+    <t>23-07-2025</t>
+  </si>
+  <si>
+    <t>OPT PAYTM 31 Jul 2025 1100 CE</t>
+  </si>
+  <si>
+    <t>24-07-2025</t>
+  </si>
+  <si>
+    <t>OPT BIOCON 31 Jul 2025 390 CE</t>
+  </si>
+  <si>
+    <t>OPT BAJAJFINSV 31 Jul 2025 2000 PE</t>
+  </si>
+  <si>
+    <t>25-07-2025</t>
+  </si>
+  <si>
+    <t>OPT APLAPOLLO 31 Jul 2025 1600 PE</t>
   </si>
   <si>
     <t>Buy Qty</t>
@@ -420,10 +438,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="34.140625" customWidth="1"/>
+    <col min="2" max="2" width="40.85546875" customWidth="1"/>
     <col min="3" max="3" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.140625" style="1"/>
   </cols>
@@ -439,10 +457,10 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="E1" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="F1" t="s">
         <v>3</v>
@@ -451,10 +469,10 @@
         <v>4</v>
       </c>
       <c r="H1" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="I1" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J1" t="s">
         <v>5</v>
@@ -477,143 +495,331 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>204</v>
+        <v>238</v>
       </c>
       <c r="B2" t="s">
         <v>11</v>
       </c>
       <c r="C2" s="1">
-        <v>45825</v>
+        <v>45859</v>
       </c>
       <c r="D2">
-        <v>75</v>
+        <v>125</v>
       </c>
       <c r="E2">
-        <v>207.45</v>
+        <v>190.9</v>
       </c>
       <c r="F2">
-        <v>15558.75</v>
+        <v>23862.5</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>12</v>
       </c>
       <c r="H2">
-        <v>75</v>
+        <v>125</v>
       </c>
       <c r="I2">
-        <v>172.8</v>
+        <v>211.55</v>
       </c>
       <c r="J2">
-        <v>12960</v>
+        <v>26443.75</v>
       </c>
       <c r="K2">
         <v>0</v>
       </c>
       <c r="L2">
-        <v>-2598.75</v>
+        <v>2581.25</v>
       </c>
       <c r="M2">
-        <v>72.819999999999993</v>
+        <v>95.51</v>
       </c>
       <c r="N2">
-        <v>-2671.57</v>
+        <v>2485.7399999999998</v>
       </c>
       <c r="O2">
-        <v>2598.75</v>
+        <v>2581.25</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>196</v>
+        <v>74</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
       </c>
       <c r="C3" s="1">
-        <v>45825</v>
+        <v>45859</v>
       </c>
       <c r="D3">
-        <v>75</v>
+        <v>325</v>
       </c>
       <c r="E3">
-        <v>155.75</v>
+        <v>72.95</v>
       </c>
       <c r="F3">
-        <v>11681.25</v>
+        <v>23708.75</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>12</v>
       </c>
       <c r="H3">
-        <v>75</v>
+        <v>325</v>
       </c>
       <c r="I3">
-        <v>146.9</v>
+        <v>83.1</v>
       </c>
       <c r="J3">
-        <v>11017.5</v>
+        <v>27007.5</v>
       </c>
       <c r="K3">
         <v>0</v>
       </c>
       <c r="L3">
-        <v>-663.75</v>
+        <v>3298.75</v>
       </c>
       <c r="M3">
-        <v>68.11</v>
+        <v>95.37</v>
       </c>
       <c r="N3">
-        <v>-731.86</v>
+        <v>3203.38</v>
       </c>
       <c r="O3">
-        <v>663.75</v>
+        <v>3298.75</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>88</v>
+        <v>225</v>
       </c>
       <c r="B4" t="s">
         <v>14</v>
       </c>
       <c r="C4" s="1">
-        <v>45826</v>
+        <v>45861</v>
       </c>
       <c r="D4">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="E4">
-        <v>139.69999999999999</v>
+        <v>40.65</v>
       </c>
       <c r="F4">
-        <v>13970</v>
+        <v>24390</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H4">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="I4">
-        <v>131</v>
+        <v>42.5</v>
       </c>
       <c r="J4">
-        <v>13100</v>
+        <v>25500</v>
       </c>
       <c r="K4">
         <v>0</v>
       </c>
       <c r="L4">
-        <v>-870</v>
+        <v>1110</v>
       </c>
       <c r="M4">
-        <v>71.59</v>
+        <v>118.78</v>
       </c>
       <c r="N4">
-        <v>-941.59</v>
+        <v>991.22</v>
       </c>
       <c r="O4">
-        <v>870</v>
+        <v>1110</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>226</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="1">
+        <v>45862</v>
+      </c>
+      <c r="D5">
+        <v>725</v>
+      </c>
+      <c r="E5">
+        <v>29.4</v>
+      </c>
+      <c r="F5">
+        <v>21315</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5">
+        <v>725</v>
+      </c>
+      <c r="I5">
+        <v>27.7</v>
+      </c>
+      <c r="J5">
+        <v>20082.5</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>-1232.5</v>
+      </c>
+      <c r="M5">
+        <v>85.32</v>
+      </c>
+      <c r="N5">
+        <v>-1317.82</v>
+      </c>
+      <c r="O5">
+        <v>1232.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>48</v>
+      </c>
+      <c r="B6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="1">
+        <v>45862</v>
+      </c>
+      <c r="D6">
+        <v>7500</v>
+      </c>
+      <c r="E6">
+        <v>14.7</v>
+      </c>
+      <c r="F6">
+        <v>110250</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6">
+        <v>7500</v>
+      </c>
+      <c r="I6">
+        <v>13.65</v>
+      </c>
+      <c r="J6">
+        <v>102375</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>-7875</v>
+      </c>
+      <c r="M6">
+        <v>289.07</v>
+      </c>
+      <c r="N6">
+        <v>-8164.07</v>
+      </c>
+      <c r="O6">
+        <v>7875</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>33</v>
+      </c>
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="1">
+        <v>45863</v>
+      </c>
+      <c r="D7">
+        <v>500</v>
+      </c>
+      <c r="E7">
+        <v>67.8</v>
+      </c>
+      <c r="F7">
+        <v>33900</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H7">
+        <v>500</v>
+      </c>
+      <c r="I7">
+        <v>77.400000000000006</v>
+      </c>
+      <c r="J7">
+        <v>38700</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <v>4800</v>
+      </c>
+      <c r="M7">
+        <v>117.53</v>
+      </c>
+      <c r="N7">
+        <v>4682.47</v>
+      </c>
+      <c r="O7">
+        <v>4800</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>15</v>
+      </c>
+      <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="1">
+        <v>45863</v>
+      </c>
+      <c r="D8">
+        <v>350</v>
+      </c>
+      <c r="E8">
+        <v>22.5</v>
+      </c>
+      <c r="F8">
+        <v>7875</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H8">
+        <v>350</v>
+      </c>
+      <c r="I8">
+        <v>22.7</v>
+      </c>
+      <c r="J8">
+        <v>7945</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="L8">
+        <v>70</v>
+      </c>
+      <c r="M8">
+        <v>62.04</v>
+      </c>
+      <c r="N8">
+        <v>7.96</v>
+      </c>
+      <c r="O8">
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>